<commit_message>
updated fig 4 and aliogned fig 1
</commit_message>
<xml_diff>
--- a/8_Data_Synthesis/Data_Extraction.xlsx
+++ b/8_Data_Synthesis/Data_Extraction.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11214"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/antoniotrovato/Documents/GitHub/RegressionTestingOptimizationSLR/8_Data_Synthesis/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\research\2026-SLR-regression-testing-optimization\8_Data_Synthesis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4704409F-B9D4-E04C-927C-102DFB175B1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B974F0A6-88CA-4A10-A9AE-A0C53BEDF5BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="620" windowWidth="28800" windowHeight="15540" xr2:uid="{FF880EED-EA60-9E49-B15D-179496B980D1}"/>
+    <workbookView xWindow="-23148" yWindow="1344" windowWidth="23256" windowHeight="13896" xr2:uid="{FF880EED-EA60-9E49-B15D-179496B980D1}"/>
   </bookViews>
   <sheets>
     <sheet name="Foglio1" sheetId="1" r:id="rId1"/>
@@ -4844,9 +4844,9 @@
     </xf>
   </cellXfs>
   <cellStyles count="3">
-    <cellStyle name="Collegamento ipertestuale" xfId="2" builtinId="8"/>
-    <cellStyle name="Normale" xfId="0" builtinId="0"/>
-    <cellStyle name="Valore non valido" xfId="1" builtinId="27"/>
+    <cellStyle name="Bad" xfId="1" builtinId="27"/>
+    <cellStyle name="Hyperlink" xfId="2" builtinId="8"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -4864,7 +4864,7 @@
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="it-IT"/>
+  <c:lang val="en-GB"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -7498,7 +7498,7 @@
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="it-IT"/>
+  <c:lang val="en-GB"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -9240,7 +9240,7 @@
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="it-IT"/>
+  <c:lang val="en-GB"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -9709,7 +9709,7 @@
 <file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="it-IT"/>
+  <c:lang val="en-GB"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -11572,7 +11572,7 @@
 <file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="it-IT"/>
+  <c:lang val="en-GB"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -13438,7 +13438,7 @@
 <file path=xl/charts/chart6.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="it-IT"/>
+  <c:lang val="en-GB"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -14219,7 +14219,7 @@
 <file path=xl/charts/chart7.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="it-IT"/>
+  <c:lang val="en-GB"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -14588,7 +14588,7 @@
 <file path=xl/charts/chart8.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="it-IT"/>
+  <c:lang val="en-GB"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -14622,6 +14622,64 @@
             <a:effectLst/>
           </c:spPr>
           <c:invertIfNegative val="0"/>
+          <c:dLbls>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:spAutoFit/>
+              </a:bodyPr>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="75000"/>
+                        <a:lumOff val="25000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:txPr>
+            <c:dLblPos val="outEnd"/>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+                <c15:leaderLines>
+                  <c:spPr>
+                    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="35000"/>
+                          <a:lumOff val="65000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:round/>
+                    </a:ln>
+                    <a:effectLst/>
+                  </c:spPr>
+                </c15:leaderLines>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
           <c:cat>
             <c:numRef>
               <c:f>Foglio1!$CN$3:$CN$15</c:f>
@@ -14740,6 +14798,64 @@
             <a:effectLst/>
           </c:spPr>
           <c:invertIfNegative val="0"/>
+          <c:dLbls>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:spAutoFit/>
+              </a:bodyPr>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="75000"/>
+                        <a:lumOff val="25000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:txPr>
+            <c:dLblPos val="outEnd"/>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+                <c15:leaderLines>
+                  <c:spPr>
+                    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="35000"/>
+                          <a:lumOff val="65000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:round/>
+                    </a:ln>
+                    <a:effectLst/>
+                  </c:spPr>
+                </c15:leaderLines>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
           <c:cat>
             <c:numRef>
               <c:f>Foglio1!$CN$3:$CN$15</c:f>
@@ -14858,6 +14974,64 @@
             <a:effectLst/>
           </c:spPr>
           <c:invertIfNegative val="0"/>
+          <c:dLbls>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:spAutoFit/>
+              </a:bodyPr>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="75000"/>
+                        <a:lumOff val="25000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:txPr>
+            <c:dLblPos val="outEnd"/>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+                <c15:leaderLines>
+                  <c:spPr>
+                    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="35000"/>
+                          <a:lumOff val="65000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:round/>
+                    </a:ln>
+                    <a:effectLst/>
+                  </c:spPr>
+                </c15:leaderLines>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
           <c:cat>
             <c:numRef>
               <c:f>Foglio1!$CN$3:$CN$15</c:f>
@@ -14961,8 +15135,9 @@
           </c:extLst>
         </c:ser>
         <c:dLbls>
+          <c:dLblPos val="outEnd"/>
           <c:showLegendKey val="0"/>
-          <c:showVal val="0"/>
+          <c:showVal val="1"/>
           <c:showCatName val="0"/>
           <c:showSerName val="0"/>
           <c:showPercent val="0"/>
@@ -19323,7 +19498,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema di Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -19640,15 +19815,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1BA3DE9A-9DC8-9B4C-920E-613E1AA78E62}">
   <dimension ref="A1:HM126"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
+  <sheetFormatPr defaultColWidth="11.19921875" defaultRowHeight="15.6"/>
   <cols>
-    <col min="27" max="27" width="22.1640625" customWidth="1"/>
-    <col min="30" max="30" width="21.1640625" customWidth="1"/>
-    <col min="32" max="32" width="8.6640625" customWidth="1"/>
-    <col min="33" max="33" width="50.1640625" customWidth="1"/>
+    <col min="27" max="27" width="22.19921875" customWidth="1"/>
+    <col min="30" max="30" width="21.19921875" customWidth="1"/>
+    <col min="32" max="32" width="8.69921875" customWidth="1"/>
+    <col min="33" max="33" width="50.19921875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:221" ht="32">
+    <row r="1" spans="1:221">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -20764,7 +20939,7 @@
         <v>0</v>
       </c>
       <c r="AS4">
-        <f t="shared" ref="AS3:AS15" si="6">SUMIF(F:F,AP4,AM:AM)</f>
+        <f t="shared" ref="AS4:AS15" si="6">SUMIF(F:F,AP4,AM:AM)</f>
         <v>2</v>
       </c>
       <c r="AT4">
@@ -21148,7 +21323,7 @@
         <v>2015</v>
       </c>
       <c r="AQ5">
-        <f t="shared" ref="AQ4:AQ15" si="8">SUMIF(F:F,AP5,AK:AK)</f>
+        <f t="shared" ref="AQ5:AQ15" si="8">SUMIF(F:F,AP5,AK:AK)</f>
         <v>8</v>
       </c>
       <c r="AR5">
@@ -27519,7 +27694,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="35" spans="1:221" ht="144">
+    <row r="35" spans="1:221" ht="115.2">
       <c r="C35" t="s">
         <v>458</v>
       </c>
@@ -27769,7 +27944,7 @@
         <v>1291</v>
       </c>
     </row>
-    <row r="37" spans="1:221" ht="112">
+    <row r="37" spans="1:221" ht="100.8">
       <c r="C37" t="s">
         <v>477</v>
       </c>
@@ -27985,7 +28160,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:221" ht="128">
+    <row r="38" spans="1:221" ht="115.2">
       <c r="C38" t="s">
         <v>486</v>
       </c>
@@ -28199,7 +28374,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:221" ht="128">
+    <row r="39" spans="1:221" ht="100.8">
       <c r="C39" t="s">
         <v>495</v>
       </c>
@@ -28413,7 +28588,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:221" ht="160">
+    <row r="40" spans="1:221" ht="144">
       <c r="C40" t="s">
         <v>504</v>
       </c>
@@ -28627,7 +28802,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:221" ht="144">
+    <row r="41" spans="1:221" ht="115.2">
       <c r="C41" t="s">
         <v>512</v>
       </c>
@@ -28841,7 +29016,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:221" ht="112">
+    <row r="42" spans="1:221" ht="100.8">
       <c r="C42" t="s">
         <v>521</v>
       </c>
@@ -29057,7 +29232,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:221" ht="80">
+    <row r="43" spans="1:221" ht="57.6">
       <c r="C43" t="s">
         <v>531</v>
       </c>
@@ -29257,7 +29432,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="1:221" ht="112">
+    <row r="44" spans="1:221" ht="100.8">
       <c r="C44" t="s">
         <v>536</v>
       </c>
@@ -29471,7 +29646,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:221" ht="192">
+    <row r="45" spans="1:221" ht="158.4">
       <c r="C45" t="s">
         <v>545</v>
       </c>
@@ -29685,7 +29860,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:221" ht="80">
+    <row r="46" spans="1:221" ht="57.6">
       <c r="C46" t="s">
         <v>556</v>
       </c>
@@ -29885,7 +30060,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:221" ht="80">
+    <row r="47" spans="1:221" ht="57.6">
       <c r="C47" t="s">
         <v>561</v>
       </c>
@@ -30085,7 +30260,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="1:221" ht="144">
+    <row r="48" spans="1:221" ht="129.6">
       <c r="C48" t="s">
         <v>565</v>
       </c>
@@ -30292,7 +30467,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="3:221" ht="144">
+    <row r="49" spans="3:221" ht="129.6">
       <c r="C49" t="s">
         <v>574</v>
       </c>
@@ -30499,7 +30674,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="3:221" ht="96">
+    <row r="50" spans="3:221" ht="86.4">
       <c r="C50" t="s">
         <v>583</v>
       </c>
@@ -30569,7 +30744,7 @@
         <v>1302</v>
       </c>
     </row>
-    <row r="51" spans="3:221" ht="96">
+    <row r="51" spans="3:221" ht="86.4">
       <c r="C51" t="s">
         <v>592</v>
       </c>
@@ -30636,7 +30811,7 @@
         <v>1266</v>
       </c>
     </row>
-    <row r="52" spans="3:221" ht="112">
+    <row r="52" spans="3:221" ht="86.4">
       <c r="C52" t="s">
         <v>600</v>
       </c>
@@ -30706,7 +30881,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="53" spans="3:221" ht="112">
+    <row r="53" spans="3:221" ht="100.8">
       <c r="C53" t="s">
         <v>609</v>
       </c>
@@ -30774,7 +30949,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="54" spans="3:221" ht="144">
+    <row r="54" spans="3:221" ht="129.6">
       <c r="C54" t="s">
         <v>618</v>
       </c>
@@ -30835,7 +31010,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="55" spans="3:221" ht="128">
+    <row r="55" spans="3:221" ht="115.2">
       <c r="C55" t="s">
         <v>626</v>
       </c>
@@ -30896,7 +31071,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="56" spans="3:221" ht="160">
+    <row r="56" spans="3:221" ht="144">
       <c r="C56" t="s">
         <v>635</v>
       </c>
@@ -30959,7 +31134,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="57" spans="3:221" ht="112">
+    <row r="57" spans="3:221" ht="100.8">
       <c r="C57" t="s">
         <v>643</v>
       </c>
@@ -31070,7 +31245,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" spans="3:221" ht="96">
+    <row r="59" spans="3:221" ht="86.4">
       <c r="C59" t="s">
         <v>656</v>
       </c>
@@ -31133,7 +31308,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="60" spans="3:221" ht="80">
+    <row r="60" spans="3:221" ht="57.6">
       <c r="C60" t="s">
         <v>664</v>
       </c>
@@ -31196,7 +31371,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="61" spans="3:221" ht="80">
+    <row r="61" spans="3:221" ht="72">
       <c r="C61" t="s">
         <v>671</v>
       </c>
@@ -31259,7 +31434,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="62" spans="3:221" ht="128">
+    <row r="62" spans="3:221" ht="115.2">
       <c r="C62" t="s">
         <v>680</v>
       </c>
@@ -31322,7 +31497,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="63" spans="3:221" ht="112">
+    <row r="63" spans="3:221" ht="100.8">
       <c r="C63" t="s">
         <v>689</v>
       </c>
@@ -31385,7 +31560,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="64" spans="3:221" ht="144">
+    <row r="64" spans="3:221" ht="115.2">
       <c r="C64" s="2" t="s">
         <v>696</v>
       </c>
@@ -31448,7 +31623,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="65" spans="1:180" ht="187">
+    <row r="65" spans="1:180" ht="140.4">
       <c r="A65" s="24">
         <v>9260075</v>
       </c>
@@ -31544,7 +31719,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="66" spans="1:180" ht="204">
+    <row r="66" spans="1:180" ht="187.2">
       <c r="A66" s="24">
         <v>8914670</v>
       </c>
@@ -31644,7 +31819,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="67" spans="1:180" ht="221">
+    <row r="67" spans="1:180" ht="187.2">
       <c r="A67" s="24">
         <v>8305938</v>
       </c>
@@ -31740,7 +31915,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="68" spans="1:180" ht="153">
+    <row r="68" spans="1:180" ht="140.4">
       <c r="A68" s="24">
         <v>8453107</v>
       </c>
@@ -31828,7 +32003,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="69" spans="1:180" ht="187">
+    <row r="69" spans="1:180" ht="124.8">
       <c r="A69" s="24">
         <v>8754416</v>
       </c>
@@ -31930,7 +32105,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="70" spans="1:180" ht="170">
+    <row r="70" spans="1:180" ht="140.4">
       <c r="A70" s="24">
         <v>7582788</v>
       </c>
@@ -32019,7 +32194,7 @@
         <v>1302</v>
       </c>
     </row>
-    <row r="71" spans="1:180" ht="153">
+    <row r="71" spans="1:180" ht="124.8">
       <c r="A71" s="24" t="s">
         <v>772</v>
       </c>
@@ -32136,7 +32311,7 @@
         <v>1301</v>
       </c>
     </row>
-    <row r="72" spans="1:180" ht="119">
+    <row r="72" spans="1:180" ht="93.6">
       <c r="A72" s="24" t="s">
         <v>790</v>
       </c>
@@ -32237,7 +32412,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="73" spans="1:180" ht="204">
+    <row r="73" spans="1:180" ht="156">
       <c r="A73" s="24" t="s">
         <v>803</v>
       </c>
@@ -32350,7 +32525,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="74" spans="1:180" ht="187">
+    <row r="74" spans="1:180" ht="171.6">
       <c r="A74" s="24" t="s">
         <v>818</v>
       </c>
@@ -32461,7 +32636,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="75" spans="1:180" ht="85">
+    <row r="75" spans="1:180" ht="78">
       <c r="A75" s="24" t="s">
         <v>831</v>
       </c>
@@ -32576,7 +32751,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="76" spans="1:180" ht="204">
+    <row r="76" spans="1:180" ht="187.2">
       <c r="A76" s="24" t="s">
         <v>844</v>
       </c>
@@ -32689,7 +32864,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="77" spans="1:180" ht="187">
+    <row r="77" spans="1:180" ht="140.4">
       <c r="A77" s="24" t="s">
         <v>856</v>
       </c>
@@ -32802,7 +32977,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="78" spans="1:180" ht="153">
+    <row r="78" spans="1:180" ht="124.8">
       <c r="A78" s="24" t="s">
         <v>872</v>
       </c>
@@ -32915,7 +33090,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="79" spans="1:180" ht="255">
+    <row r="79" spans="1:180" ht="202.8">
       <c r="A79" s="24" t="s">
         <v>884</v>
       </c>
@@ -33020,7 +33195,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="80" spans="1:180" ht="187">
+    <row r="80" spans="1:180" ht="140.4">
       <c r="A80" s="24" t="s">
         <v>895</v>
       </c>
@@ -33133,7 +33308,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="81" spans="1:180" ht="187">
+    <row r="81" spans="1:180" ht="156">
       <c r="A81" s="24" t="s">
         <v>909</v>
       </c>
@@ -33246,7 +33421,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="82" spans="1:180" ht="170">
+    <row r="82" spans="1:180" ht="124.8">
       <c r="A82" s="24"/>
       <c r="B82" s="25"/>
       <c r="C82" s="26" t="s">
@@ -33327,7 +33502,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="83" spans="1:180" ht="187">
+    <row r="83" spans="1:180" ht="140.4">
       <c r="A83" s="24"/>
       <c r="B83" s="25"/>
       <c r="C83" s="26" t="s">
@@ -33422,7 +33597,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="84" spans="1:180" ht="187">
+    <row r="84" spans="1:180" ht="171.6">
       <c r="A84" s="24"/>
       <c r="B84" s="25"/>
       <c r="C84" s="26" t="s">
@@ -33517,7 +33692,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="85" spans="1:180" ht="170">
+    <row r="85" spans="1:180" ht="124.8">
       <c r="A85" s="24"/>
       <c r="B85" s="25"/>
       <c r="C85" s="26" t="s">
@@ -33603,7 +33778,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="86" spans="1:180" ht="102">
+    <row r="86" spans="1:180" ht="78">
       <c r="A86" s="24"/>
       <c r="B86" s="25"/>
       <c r="C86" s="26" t="s">
@@ -33673,7 +33848,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="87" spans="1:180" ht="136">
+    <row r="87" spans="1:180" ht="124.8">
       <c r="A87" s="24"/>
       <c r="B87" s="25"/>
       <c r="C87" s="26" t="s">
@@ -33743,7 +33918,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="88" spans="1:180" ht="153">
+    <row r="88" spans="1:180" ht="109.2">
       <c r="A88" s="24"/>
       <c r="B88" s="25"/>
       <c r="C88" s="26" t="s">
@@ -33813,7 +33988,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="89" spans="1:180" ht="136">
+    <row r="89" spans="1:180" ht="109.2">
       <c r="A89" s="24"/>
       <c r="B89" s="25"/>
       <c r="C89" s="26" t="s">
@@ -33983,7 +34158,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="91" spans="1:180" ht="153">
+    <row r="91" spans="1:180" ht="124.8">
       <c r="A91" s="24"/>
       <c r="B91" s="25"/>
       <c r="C91" s="26" t="s">
@@ -34067,7 +34242,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="92" spans="1:180" ht="372">
+    <row r="92" spans="1:180" ht="327.60000000000002">
       <c r="A92" s="24"/>
       <c r="B92" s="25"/>
       <c r="C92" s="26" t="s">
@@ -34151,7 +34326,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="93" spans="1:180" ht="102">
+    <row r="93" spans="1:180" ht="78">
       <c r="A93" s="24"/>
       <c r="B93" s="25"/>
       <c r="C93" s="26" t="s">
@@ -34221,7 +34396,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="94" spans="1:180" ht="153">
+    <row r="94" spans="1:180" ht="140.4">
       <c r="A94" s="24"/>
       <c r="B94" s="25"/>
       <c r="C94" s="26" t="s">
@@ -34305,7 +34480,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="95" spans="1:180" ht="119">
+    <row r="95" spans="1:180" ht="109.2">
       <c r="A95" s="24"/>
       <c r="B95" s="25"/>
       <c r="C95" s="26" t="s">
@@ -37023,7 +37198,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1B91C968-CFFD-1A41-862E-46C430B19788}">
   <dimension ref="A1:E1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
+  <sheetFormatPr defaultColWidth="11.19921875" defaultRowHeight="15.6"/>
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" s="32"/>

</xml_diff>